<commit_message>
Presentación V3: reordenar diapositivas (situación original → RUP y UML → resultado)
Solo cambia el orden, sin tocar textos, diagramas ni notas: el bloque de
la web renovada (antes 7–11) pasa a 20–24. Se ajustan la numeración de
secciones y las referencias a diapositivas en la guía, los anexos y el
informe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bgTV8cWdz9SLoTLCZtcCS
</commit_message>
<xml_diff>
--- a/RUP_BLACK_HAWK/ANEXOS/BLACK_HAWK_RUP_ANEXOS_V3.xlsx
+++ b/RUP_BLACK_HAWK/ANEXOS/BLACK_HAWK_RUP_ANEXOS_V3.xlsx
@@ -7952,7 +7952,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Presentación V3 diap. 20; monografía V3</t>
+          <t>Presentación V3 diap. 15; monografía V3</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Presentación V3 diap. 21; monografía V3</t>
+          <t>Presentación V3 diap. 16; monografía V3</t>
         </is>
       </c>
     </row>
@@ -8006,7 +8006,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Presentación V3 diap. 22; monografía V3</t>
+          <t>Presentación V3 diap. 17; monografía V3</t>
         </is>
       </c>
     </row>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Presentación V3 diap. 23; monografía V3</t>
+          <t>Presentación V3 diap. 18; monografía V3</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8060,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Presentación V3 diap. 24; monografía V3</t>
+          <t>Presentación V3 diap. 19; monografía V3</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Diapositivas 4 y 8</t>
+          <t>Diapositivas 4 y 21</t>
         </is>
       </c>
     </row>
@@ -8547,7 +8547,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Diapositiva 8</t>
+          <t>Diapositiva 21</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Diapositivas 11 y 16</t>
+          <t>Diapositivas 11 y 24</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Diapositiva 11</t>
+          <t>Diapositiva 24</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Diapositivas 10 y 22</t>
+          <t>Diapositivas 17 y 23</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Diapositivas 10 y 11</t>
+          <t>Diapositivas 23 y 24</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Diapositivas 19 y 25</t>
+          <t>Diapositivas 14 y 25</t>
         </is>
       </c>
     </row>
@@ -8709,7 +8709,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Diapositivas 19 y 25</t>
+          <t>Diapositivas 14 y 25</t>
         </is>
       </c>
     </row>
@@ -8736,7 +8736,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Diapositivas 19 y 25</t>
+          <t>Diapositivas 14 y 25</t>
         </is>
       </c>
     </row>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Diapositivas 14–18</t>
+          <t>Diapositivas 9–13</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9383,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9569,7 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -9755,7 +9755,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -9817,7 +9817,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -10189,7 +10189,7 @@
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -10251,7 +10251,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -10871,7 +10871,7 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -11286,7 +11286,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>
@@ -11580,7 +11580,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Sí (diap. 19)</t>
+          <t>Sí (diap. 14)</t>
         </is>
       </c>
     </row>

</xml_diff>